<commit_message>
Agregar ingesta de permisos de construccion (F79), con supresion de barrios bajo el umbral
</commit_message>
<xml_diff>
--- a/entrega1/Diccionario_de_datos_TallerDatos.xlsx
+++ b/entrega1/Diccionario_de_datos_TallerDatos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nsald\Documents\Cerebro Orlando\entrega1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50442504-CC82-4FE2-85C1-1822759050F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3C6ABA-D0B7-4357-B238-05BCA9072C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1785" uniqueCount="822">
   <si>
     <t>Taller de datos · Entrega 1 · El lago y su diccionario</t>
   </si>
@@ -2485,6 +2485,27 @@
   </si>
   <si>
     <t>1978-Q2 a 2026-Q2 (193 trimestres)</t>
+  </si>
+  <si>
+    <t>F106</t>
+  </si>
+  <si>
+    <t>Casos de la Policía de Orlando (OPD Cases Viewing, capa LERMSCases4Dashboard)</t>
+  </si>
+  <si>
+    <t>https://gis.orlando.gov/server/rest/services/OPD_Cases_Viewing/FeatureServer/0/query?where=1%3D1&amp;outFields=*&amp;f=geojson</t>
+  </si>
+  <si>
+    <t>Ciudad de Orlando, por punto; 126 barrios (campo NeighborhoodName)</t>
+  </si>
+  <si>
+    <t>2021-02-13 a 2026-10-05</t>
+  </si>
+  <si>
+    <t>Búsqueda asistida por IA (Claude): enlace «View the OPD Crime &amp; Cases Dashboard» de orlando.gov/Public-Safety/OPD/OPD-Records-Open-Data → tablero ArcGIS (orl.maps.arcgis.com, item eae3bde08de34ea0b7c2a637b255b48b) → capa del servicio</t>
+  </si>
+  <si>
+    <t>Prioridad alta. No está en el portal de datos abiertos (F01, F79 a F105): es la capa que alimenta el tablero de casos de la OPD. Prueba 2026-10-06 (script de Claude): HTTP 200, JSON; 239.996 casos con geometría de punto; 91 tipos de caso; 126 barrios y 5.731 casos sin barrio; campos CaseNumber, CaseDate, CaseType, CommDistID, Beat, Sector, Division, NeighborhoodName. Sin licencia: el campo licenseInfo del tablero y del mapa está vacío y la capa no trae copyrightText. Consulta máxima de 2.000 registros por llamada (hay que paginar). Personas: no trae nombres, pero el número de caso, la fecha y el punto exacto pueden identificar a víctimas o domicilios. Si se integra, solo conteos por barrio y mes, sin CaseNumber ni coordenadas. Los avisos legales de orlando.gov prohíben el uso comercial sin permiso (ver F02).</t>
   </si>
 </sst>
 </file>
@@ -2633,7 +2654,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2669,6 +2690,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5921,16 +5945,16 @@
       <c r="G61" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="H61" s="12" t="s">
+      <c r="H61" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="I61" s="12" t="s">
+      <c r="I61" s="11" t="s">
         <v>49</v>
       </c>
       <c r="J61" s="11" t="s">
         <v>455</v>
       </c>
-      <c r="K61" s="12" t="s">
+      <c r="K61" s="11" t="s">
         <v>456</v>
       </c>
       <c r="L61" s="12" t="s">
@@ -5990,7 +6014,7 @@
         <v>65</v>
       </c>
       <c r="N62" s="11" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="O62" s="11" t="s">
         <v>465</v>
@@ -6574,7 +6598,7 @@
         <v>65</v>
       </c>
       <c r="N74" s="11" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="O74" s="11" t="s">
         <v>546</v>
@@ -6624,7 +6648,7 @@
         <v>65</v>
       </c>
       <c r="N75" s="11" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="O75" s="11" t="s">
         <v>552</v>
@@ -7466,7 +7490,7 @@
         <v>65</v>
       </c>
       <c r="N92" s="11" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="O92" s="11" t="s">
         <v>608</v>
@@ -7566,7 +7590,7 @@
         <v>65</v>
       </c>
       <c r="N94" s="11" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="O94" s="11" t="s">
         <v>608</v>
@@ -7766,7 +7790,7 @@
         <v>65</v>
       </c>
       <c r="N98" s="11" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="O98" s="11" t="s">
         <v>608</v>
@@ -8326,22 +8350,54 @@
       </c>
     </row>
     <row r="110" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="11"/>
-      <c r="B110" s="11"/>
-      <c r="C110" s="11"/>
-      <c r="D110" s="11"/>
-      <c r="E110" s="11"/>
-      <c r="F110" s="11"/>
-      <c r="G110" s="12"/>
-      <c r="H110" s="11"/>
-      <c r="I110" s="12"/>
-      <c r="J110" s="11"/>
-      <c r="K110" s="12"/>
-      <c r="L110" s="12"/>
-      <c r="M110" s="11"/>
-      <c r="N110" s="11"/>
-      <c r="O110" s="11"/>
-      <c r="P110" s="11"/>
+      <c r="A110" s="11" t="s">
+        <v>815</v>
+      </c>
+      <c r="B110" s="11" t="s">
+        <v>816</v>
+      </c>
+      <c r="C110" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D110" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E110" s="11" t="s">
+        <v>817</v>
+      </c>
+      <c r="F110" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="G110" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H110" s="11" t="s">
+        <v>606</v>
+      </c>
+      <c r="I110" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="J110" s="11" t="s">
+        <v>818</v>
+      </c>
+      <c r="K110" s="12" t="s">
+        <v>819</v>
+      </c>
+      <c r="L110" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="M110" s="17">
+        <v>46301</v>
+      </c>
+      <c r="N110" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="O110" s="11" t="s">
+        <v>820</v>
+      </c>
+      <c r="P110" s="11" t="s">
+        <v>821</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="6">
@@ -8357,7 +8413,7 @@
       <formula1>"API sin llave,API con llave gratuita,Descarga directa,Solo PDF o página,Bloquea scripts o pide sesión"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" error="Elijan una opción de la lista" sqref="I5:I110" xr:uid="{00000000-0002-0000-0100-000003000000}">
+    <dataValidation type="list" allowBlank="1" error="Elijan una opción de la lista" sqref="I5:I60 I62:I110" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>"No,Solo conteos por zona,Personas identificables,Texto libre sin revisar"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9698,7 +9754,7 @@
       </c>
       <c r="B4" s="14">
         <f>COUNTA('1. Fuentes'!A5:A110)</f>
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9707,7 +9763,7 @@
       </c>
       <c r="B5" s="14">
         <f>COUNTIF('1. Fuentes'!N5:N110,"Integrada al lago")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9716,7 +9772,7 @@
       </c>
       <c r="B6" s="14">
         <f>COUNTIF('1. Fuentes'!N5:N110,"Candidata")</f>
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9752,7 +9808,7 @@
       </c>
       <c r="B10" s="14">
         <f>COUNTIF('1. Fuentes'!H5:H110,"no declara")+COUNTIFS('1. Fuentes'!A5:A110,"&lt;&gt;",'1. Fuentes'!H5:H110,"")</f>
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9761,7 +9817,7 @@
       </c>
       <c r="B11" s="14">
         <f>COUNTIF('1. Fuentes'!I5:I110,"Personas identificables")+COUNTIF('1. Fuentes'!I5:I110,"Texto libre sin revisar")</f>
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>